<commit_message>
fixed traj with updated answers
</commit_message>
<xml_diff>
--- a/Data_logs_final.xlsx
+++ b/Data_logs_final.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\KAUST\MCTA_Final\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\KAUST\med_agent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C53E64D-E6A7-4889-89D9-341F43438C4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{078BA8AC-342D-4E9B-997E-B4A687566B40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27375,7 +27375,7 @@
       <c r="V1000" s="10"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C6:C20 F6:I20 D6:E100 H28:I28 B108:B109 D108:D128 B182:B223 B6:B100">
+  <conditionalFormatting sqref="C6:C20 F6:I20 B6:B100 D6:E100 H28:I28 B108:B109 D108:D128 B182:B223">
     <cfRule type="expression" dxfId="3" priority="9">
       <formula>#REF!="Yes"</formula>
     </cfRule>
@@ -27407,7 +27407,7 @@
   <sheetFormatPr defaultRowHeight="27"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="42"/>
-    <col min="2" max="2" width="26" style="42" customWidth="1"/>
+    <col min="2" max="2" width="58" style="42" customWidth="1"/>
     <col min="3" max="3" width="25" style="42" customWidth="1"/>
     <col min="4" max="4" width="28.88671875" style="42" customWidth="1"/>
     <col min="5" max="5" width="23" style="42" customWidth="1"/>
@@ -27446,7 +27446,7 @@
       <c r="G3" s="47"/>
       <c r="H3" s="47"/>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" ht="54">
       <c r="A4" s="48" t="s">
         <v>0</v>
       </c>
@@ -27560,7 +27560,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="297">
+    <row r="9" spans="1:8" ht="324">
       <c r="A9" s="49">
         <v>5</v>
       </c>
@@ -27629,7 +27629,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="108">
+    <row r="12" spans="1:8" ht="135">
       <c r="A12" s="49">
         <v>8</v>
       </c>

</xml_diff>